<commit_message>
fix: correct CMRb/CMRs/CPTA speed ranges and stop NM_04 double-flagging speed
Audited every scenario family's vut_speed_range_kmh against the EuroNCAP Frontal
v1.1 speed matrices. Three were wrong and false-FAILed valid scenarios:
  CMRb [30,80]->[30,130]  (Standard 30-80 + Extended 90-130)
  CMRs [10,50]->[10,80]   (AEB 10-50 + FCW 60-80)
  CPTA + fo/fs/no/ns [10,60]->[10,25]  (VUT turning speed; 60 was a stale default)
The other 26 families match the protocol. config.xlsx regenerated (round-trips).

CH_NM_04 no longer re-checks the VUT speed range that CH_SC_18 already owns, so a
single out-of-range speed is not double-reported as two failures.
</commit_message>
<xml_diff>
--- a/config.xlsx
+++ b/config.xlsx
@@ -1501,7 +1501,7 @@
         <v>10</v>
       </c>
       <c r="D13" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -1525,7 +1525,7 @@
         <v>10</v>
       </c>
       <c r="D14" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -1549,7 +1549,7 @@
         <v>10</v>
       </c>
       <c r="D15" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -1573,7 +1573,7 @@
         <v>10</v>
       </c>
       <c r="D16" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -1597,7 +1597,7 @@
         <v>10</v>
       </c>
       <c r="D17" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -1885,7 +1885,7 @@
         <v>10</v>
       </c>
       <c r="D29" t="n">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1909,7 +1909,7 @@
         <v>30</v>
       </c>
       <c r="D30" t="n">
-        <v>80</v>
+        <v>130</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>

</xml_diff>